<commit_message>
Update index.html and schedule files for Oncoderma 2026
- Changed registration links to indicate that registrations are closed in index.html.
- Updated speaker details for the session "Manejo na nova era de tratamento do melanoma: novos desafios" in programacao-preliminar-2026.csv.
- Adjusted related content in the backup schedule files to reflect the latest changes.
</commit_message>
<xml_diff>
--- a/oncoderma2026/schedule/programacao-preliminar-2026.xlsx
+++ b/oncoderma2026/schedule/programacao-preliminar-2026.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="19425" windowHeight="10305" activeTab="3"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="19425" windowHeight="10305" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Programação " sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="196">
   <si>
     <t xml:space="preserve">Abertura </t>
   </si>
@@ -639,22 +639,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">MESA 5 — MANEJO NA NOVA ERA DE TRATAMENTO DO MELANOMA: NOVOS DESAFIOS
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Presidente: Luciana Câmara
-Debatedores: Antônio de Pádua, Heberton Medeiros</t>
-    </r>
-  </si>
-  <si>
     <t>Cirurgião oncológico pelo Ac Camargo Câncer Center
 Doutor em Oncologia/Melanoma pelo Ac camargo câncer Center/SP
 Coordenador da oncologia cutânea da clínico Unionco Pró-Pele, Clínica RICO e Hospital Barão de Lucena                                                                                                                                                                   Membro fundador - Clube da Pele de Pernambuco.
@@ -961,12 +945,31 @@
 Debatedores: Manoel Andrade, Domingo Lins</t>
     </r>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">MESA 5 — MANEJO NA NOVA ERA DE TRATAMENTO DO MELANOMA: NOVOS DESAFIOS
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Presidente: Luciana Câmara
+Debatedores: Antônio de Pádua, Silvia Fontan</t>
+    </r>
+  </si>
+  <si>
+    <t>não vai poder participar</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1101,8 +1104,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFFFF00"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1143,6 +1152,12 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1367,7 +1382,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1607,76 +1622,71 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="5" fillId="3" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="3" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="3" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="4" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="4" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="3" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="4" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="3" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="3" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1722,7 +1732,7 @@
         <xdr:cNvPr id="2" name="Imagem 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E9285274-1F62-44A0-86B5-0A9C05063892}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{E9285274-1F62-44A0-86B5-0A9C05063892}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1765,7 +1775,7 @@
         <xdr:cNvPr id="3" name="Imagem 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{59D4BE7A-9C66-4A19-B8CF-BD13EB1FF6CA}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{59D4BE7A-9C66-4A19-B8CF-BD13EB1FF6CA}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1777,7 +1787,7 @@
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" val="0"/>
             </a:ext>
           </a:extLst>
         </a:blip>
@@ -1797,7 +1807,7 @@
         <a:noFill/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -1826,7 +1836,7 @@
         <xdr:cNvPr id="4" name="Imagem 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B70868BB-961B-45D7-83FD-83FD19251BFB}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{B70868BB-961B-45D7-83FD-83FD19251BFB}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1838,7 +1848,7 @@
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" val="0"/>
             </a:ext>
           </a:extLst>
         </a:blip>
@@ -1876,7 +1886,7 @@
         <xdr:cNvPr id="5" name="Imagem 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6775E892-588D-4321-89FA-830E0E3FCFB6}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{6775E892-588D-4321-89FA-830E0E3FCFB6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1888,7 +1898,7 @@
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" val="0"/>
             </a:ext>
           </a:extLst>
         </a:blip>
@@ -2207,11 +2217,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="16" customFormat="1" ht="45" customHeight="1">
-      <c r="A1" s="96" t="s">
+      <c r="A1" s="91" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="97"/>
-      <c r="C1" s="97"/>
+      <c r="B1" s="92"/>
+      <c r="C1" s="92"/>
     </row>
     <row r="2" spans="1:4" ht="18" customHeight="1">
       <c r="A2" s="17" t="s">
@@ -2226,10 +2236,10 @@
       <c r="A3" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="98" t="s">
+      <c r="B3" s="93" t="s">
         <v>135</v>
       </c>
-      <c r="C3" s="98"/>
+      <c r="C3" s="93"/>
     </row>
     <row r="4" spans="1:4" ht="27" customHeight="1">
       <c r="A4" s="3" t="s">
@@ -2277,10 +2287,10 @@
       <c r="A8" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="B8" s="95" t="s">
-        <v>142</v>
-      </c>
-      <c r="C8" s="95"/>
+      <c r="B8" s="96" t="s">
+        <v>141</v>
+      </c>
+      <c r="C8" s="96"/>
     </row>
     <row r="9" spans="1:4" ht="27" customHeight="1">
       <c r="A9" s="9" t="s">
@@ -2339,19 +2349,19 @@
       <c r="A14" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="100" t="s">
+      <c r="B14" s="95" t="s">
         <v>2</v>
       </c>
-      <c r="C14" s="100"/>
+      <c r="C14" s="95"/>
     </row>
     <row r="15" spans="1:4" ht="45" customHeight="1">
       <c r="A15" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="B15" s="99" t="s">
+      <c r="B15" s="94" t="s">
         <v>137</v>
       </c>
-      <c r="C15" s="99"/>
+      <c r="C15" s="94"/>
     </row>
     <row r="16" spans="1:4" ht="27" customHeight="1">
       <c r="A16" s="9" t="s">
@@ -2385,7 +2395,7 @@
         <v>43</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D18" s="1"/>
     </row>
@@ -2399,13 +2409,13 @@
       <c r="C19" s="15"/>
     </row>
     <row r="20" spans="1:4" ht="45" customHeight="1">
-      <c r="A20" s="112" t="s">
+      <c r="A20" s="90" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="111" t="s">
+      <c r="B20" s="99" t="s">
         <v>138</v>
       </c>
-      <c r="C20" s="111"/>
+      <c r="C20" s="99"/>
       <c r="D20" s="28"/>
     </row>
     <row r="21" spans="1:4" ht="27" customHeight="1">
@@ -2455,10 +2465,10 @@
       <c r="A25" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="B25" s="95" t="s">
-        <v>139</v>
-      </c>
-      <c r="C25" s="95"/>
+      <c r="B25" s="96" t="s">
+        <v>194</v>
+      </c>
+      <c r="C25" s="96"/>
     </row>
     <row r="26" spans="1:4" ht="27" customHeight="1">
       <c r="A26" s="9" t="s">
@@ -2506,19 +2516,19 @@
       <c r="A30" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B30" s="93" t="s">
+      <c r="B30" s="97" t="s">
         <v>2</v>
       </c>
-      <c r="C30" s="94"/>
+      <c r="C30" s="98"/>
     </row>
     <row r="31" spans="1:4" ht="45" customHeight="1">
       <c r="A31" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B31" s="95" t="s">
-        <v>194</v>
-      </c>
-      <c r="C31" s="95"/>
+      <c r="B31" s="96" t="s">
+        <v>193</v>
+      </c>
+      <c r="C31" s="96"/>
     </row>
     <row r="32" spans="1:4" ht="27" customHeight="1">
       <c r="A32" s="9" t="s">
@@ -2578,10 +2588,10 @@
       <c r="A37" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="B37" s="95" t="s">
+      <c r="B37" s="96" t="s">
         <v>90</v>
       </c>
-      <c r="C37" s="95"/>
+      <c r="C37" s="96"/>
     </row>
     <row r="38" spans="1:4" ht="27" customHeight="1">
       <c r="A38" s="9" t="s">
@@ -2613,7 +2623,7 @@
         <v>47</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="27" customHeight="1">
@@ -2636,16 +2646,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B25:C25"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B25:C25"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" scale="98" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -2676,7 +2686,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="82" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D1" s="82" t="s">
         <v>92</v>
@@ -2690,7 +2700,7 @@
         <v>94</v>
       </c>
       <c r="C2" s="37" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D2" s="37" t="s">
         <v>95</v>
@@ -2704,7 +2714,7 @@
         <v>70</v>
       </c>
       <c r="C3" s="37" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D3" s="37" t="s">
         <v>100</v>
@@ -2718,7 +2728,7 @@
         <v>98</v>
       </c>
       <c r="C4" s="37" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D4" s="37" t="s">
         <v>136</v>
@@ -2732,7 +2742,7 @@
         <v>105</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D5" s="37" t="s">
         <v>107</v>
@@ -2746,7 +2756,7 @@
         <v>108</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D6" s="37" t="s">
         <v>109</v>
@@ -2760,10 +2770,10 @@
         <v>81</v>
       </c>
       <c r="C7" s="46" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D7" s="46" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="66" customFormat="1" ht="90.75" customHeight="1">
@@ -2774,7 +2784,7 @@
         <v>112</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D8" s="37" t="s">
         <v>113</v>
@@ -2788,7 +2798,7 @@
         <v>69</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D9" s="37" t="s">
         <v>99</v>
@@ -2802,7 +2812,7 @@
         <v>104</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D10" s="37" t="s">
         <v>114</v>
@@ -2816,10 +2826,10 @@
         <v>78</v>
       </c>
       <c r="C11" s="74" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D11" s="74" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="66" customFormat="1" ht="41.25" customHeight="1">
@@ -2830,10 +2840,10 @@
         <v>89</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D12" s="77" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E12" s="80"/>
     </row>
@@ -2842,13 +2852,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="37" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C13" s="37" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D13" s="77" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E13" s="80"/>
     </row>
@@ -2860,7 +2870,7 @@
         <v>79</v>
       </c>
       <c r="C14" s="71" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D14" s="71" t="s">
         <v>111</v>
@@ -2874,10 +2884,10 @@
         <v>110</v>
       </c>
       <c r="C15" s="37" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D15" s="37" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="60" customHeight="1">
@@ -2888,10 +2898,10 @@
         <v>88</v>
       </c>
       <c r="C16" s="46" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D16" s="47" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="66" customFormat="1" ht="48.75" customHeight="1">
@@ -2902,7 +2912,7 @@
         <v>71</v>
       </c>
       <c r="C17" s="74" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D17" s="74" t="s">
         <v>101</v>
@@ -2913,13 +2923,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="46" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C18" s="46" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D18" s="74" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E18" s="79"/>
     </row>
@@ -2931,7 +2941,7 @@
         <v>96</v>
       </c>
       <c r="C19" s="37" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D19" s="37" t="s">
         <v>97</v>
@@ -2945,7 +2955,7 @@
         <v>75</v>
       </c>
       <c r="C20" s="37" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D20" s="37" t="s">
         <v>106</v>
@@ -2959,7 +2969,7 @@
         <v>102</v>
       </c>
       <c r="C21" s="37" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D21" s="37" t="s">
         <v>103</v>
@@ -2973,10 +2983,10 @@
         <v>72</v>
       </c>
       <c r="C22" s="37" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D22" s="59" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E22" s="80"/>
     </row>
@@ -2988,7 +2998,7 @@
         <v>64</v>
       </c>
       <c r="C23" s="37" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D23" s="37" t="s">
         <v>93</v>
@@ -3002,10 +3012,10 @@
         <v>67</v>
       </c>
       <c r="C24" s="37" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D24" s="37" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E24" s="80"/>
     </row>
@@ -3043,7 +3053,7 @@
         <v>122</v>
       </c>
       <c r="B2" s="69" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="34" customFormat="1" ht="61.5" customHeight="1">
@@ -3059,10 +3069,10 @@
         <v>125</v>
       </c>
       <c r="B4" s="73" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C4" s="76" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="34" customFormat="1" ht="49.5" customHeight="1">
@@ -3091,10 +3101,10 @@
     </row>
     <row r="8" spans="1:3" ht="63.75" customHeight="1">
       <c r="A8" s="43" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B8" s="74" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C8" s="75"/>
     </row>
@@ -3103,16 +3113,19 @@
         <v>133</v>
       </c>
       <c r="B9" s="74" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C9" s="76"/>
     </row>
     <row r="10" spans="1:3" ht="36" customHeight="1">
-      <c r="A10" s="40" t="s">
+      <c r="A10" s="110" t="s">
         <v>134</v>
       </c>
-      <c r="B10" s="46" t="s">
-        <v>141</v>
+      <c r="B10" s="111" t="s">
+        <v>140</v>
+      </c>
+      <c r="C10" s="75" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="11" spans="1:3" s="34" customFormat="1" ht="32.25" customHeight="1">
@@ -3120,7 +3133,7 @@
         <v>123</v>
       </c>
       <c r="B11" s="74" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12" spans="1:3" s="34" customFormat="1" ht="147.75" customHeight="1">
@@ -3128,16 +3141,16 @@
         <v>121</v>
       </c>
       <c r="B12" s="59" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C12" s="76"/>
     </row>
     <row r="13" spans="1:3" s="34" customFormat="1" ht="100.5" customHeight="1">
       <c r="A13" s="36" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B13" s="37" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C13" s="76"/>
     </row>
@@ -3163,6 +3176,7 @@
     <sortCondition ref="A1"/>
   </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3183,28 +3197,28 @@
   <sheetData>
     <row r="1" spans="1:9" s="52" customFormat="1">
       <c r="B1" s="53" t="s">
+        <v>145</v>
+      </c>
+      <c r="C1" s="52" t="s">
         <v>146</v>
       </c>
-      <c r="C1" s="52" t="s">
+      <c r="D1" s="67" t="s">
         <v>147</v>
       </c>
-      <c r="D1" s="67" t="s">
+      <c r="E1" s="67" t="s">
         <v>148</v>
       </c>
-      <c r="E1" s="67" t="s">
+      <c r="F1" s="67" t="s">
         <v>149</v>
       </c>
-      <c r="F1" s="67" t="s">
+      <c r="G1" s="52" t="s">
         <v>150</v>
       </c>
-      <c r="G1" s="52" t="s">
+      <c r="H1" s="52" t="s">
         <v>151</v>
       </c>
-      <c r="H1" s="52" t="s">
+      <c r="I1" s="52" t="s">
         <v>152</v>
-      </c>
-      <c r="I1" s="52" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="45">
@@ -3215,19 +3229,19 @@
         <v>94</v>
       </c>
       <c r="C2" s="49" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D2" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E2" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F2" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G2" s="50" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H2" s="55" t="s">
         <v>10</v>
@@ -3244,73 +3258,73 @@
         <v>122</v>
       </c>
       <c r="C3" s="49" t="s">
+        <v>155</v>
+      </c>
+      <c r="D3" s="57" t="s">
+        <v>167</v>
+      </c>
+      <c r="E3" s="57" t="s">
+        <v>167</v>
+      </c>
+      <c r="F3" s="57" t="s">
+        <v>167</v>
+      </c>
+      <c r="G3" s="50" t="s">
         <v>156</v>
-      </c>
-      <c r="D3" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="E3" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="F3" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="G3" s="50" t="s">
-        <v>157</v>
       </c>
       <c r="H3" s="60" t="s">
         <v>8</v>
       </c>
       <c r="I3" s="50" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="45">
-      <c r="A4" s="103">
+      <c r="A4" s="106">
         <v>3</v>
       </c>
-      <c r="B4" s="105" t="s">
+      <c r="B4" s="104" t="s">
         <v>119</v>
       </c>
       <c r="C4" s="49" t="s">
-        <v>160</v>
-      </c>
-      <c r="D4" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="E4" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="F4" s="101" t="s">
-        <v>168</v>
+        <v>159</v>
+      </c>
+      <c r="D4" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="E4" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="F4" s="100" t="s">
+        <v>167</v>
       </c>
       <c r="G4" s="50" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H4" s="61" t="s">
         <v>83</v>
       </c>
       <c r="I4" s="50" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="60">
-      <c r="A5" s="104"/>
-      <c r="B5" s="106"/>
+      <c r="A5" s="107"/>
+      <c r="B5" s="105"/>
       <c r="C5" s="49" t="s">
-        <v>156</v>
-      </c>
-      <c r="D5" s="102"/>
-      <c r="E5" s="102"/>
-      <c r="F5" s="102"/>
+        <v>155</v>
+      </c>
+      <c r="D5" s="101"/>
+      <c r="E5" s="101"/>
+      <c r="F5" s="101"/>
       <c r="G5" s="50" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H5" s="61" t="s">
         <v>18</v>
       </c>
       <c r="I5" s="50" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="60">
@@ -3321,19 +3335,19 @@
         <v>70</v>
       </c>
       <c r="C6" s="49" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D6" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E6" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F6" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G6" s="50" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H6" s="58" t="s">
         <v>52</v>
@@ -3350,19 +3364,19 @@
         <v>98</v>
       </c>
       <c r="C7" s="49" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D7" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E7" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F7" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G7" s="50" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H7" s="58" t="s">
         <v>50</v>
@@ -3379,23 +3393,23 @@
         <v>125</v>
       </c>
       <c r="C8" s="49" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D8" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E8" s="57"/>
       <c r="F8" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G8" s="50" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H8" s="60" t="s">
         <v>84</v>
       </c>
       <c r="I8" s="50" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="45">
@@ -3406,19 +3420,19 @@
         <v>105</v>
       </c>
       <c r="C9" s="49" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D9" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E9" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F9" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G9" s="50" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H9" s="58" t="s">
         <v>34</v>
@@ -3435,67 +3449,67 @@
         <v>128</v>
       </c>
       <c r="C10" s="49" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D10" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E10" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F10" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G10" s="50" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H10" s="63" t="s">
         <v>61</v>
       </c>
       <c r="I10" s="50" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="45">
-      <c r="A11" s="103">
+      <c r="A11" s="106">
         <v>9</v>
       </c>
-      <c r="B11" s="109" t="s">
+      <c r="B11" s="102" t="s">
         <v>115</v>
       </c>
       <c r="C11" s="49" t="s">
-        <v>155</v>
-      </c>
-      <c r="D11" s="107" t="s">
-        <v>168</v>
-      </c>
-      <c r="E11" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="F11" s="101" t="s">
-        <v>168</v>
+        <v>154</v>
+      </c>
+      <c r="D11" s="108" t="s">
+        <v>167</v>
+      </c>
+      <c r="E11" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="F11" s="100" t="s">
+        <v>167</v>
       </c>
       <c r="G11" s="50" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H11" s="64" t="s">
         <v>8</v>
       </c>
       <c r="I11" s="50" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="45">
-      <c r="A12" s="104"/>
-      <c r="B12" s="110"/>
+      <c r="A12" s="107"/>
+      <c r="B12" s="103"/>
       <c r="C12" s="49" t="s">
-        <v>156</v>
-      </c>
-      <c r="D12" s="108"/>
-      <c r="E12" s="102"/>
-      <c r="F12" s="102"/>
+        <v>155</v>
+      </c>
+      <c r="D12" s="109"/>
+      <c r="E12" s="101"/>
+      <c r="F12" s="101"/>
       <c r="G12" s="50" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H12" s="58" t="s">
         <v>56</v>
@@ -3512,67 +3526,67 @@
         <v>131</v>
       </c>
       <c r="C13" s="49" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D13" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E13" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F13" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G13" s="50" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H13" s="63" t="s">
         <v>61</v>
       </c>
       <c r="I13" s="50" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="45">
-      <c r="A14" s="103">
+      <c r="A14" s="106">
         <v>11</v>
       </c>
-      <c r="B14" s="105" t="s">
+      <c r="B14" s="104" t="s">
         <v>108</v>
       </c>
       <c r="C14" s="49" t="s">
-        <v>156</v>
-      </c>
-      <c r="D14" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="E14" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="F14" s="101" t="s">
-        <v>168</v>
+        <v>155</v>
+      </c>
+      <c r="D14" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="E14" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="F14" s="100" t="s">
+        <v>167</v>
       </c>
       <c r="G14" s="50" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H14" s="65" t="s">
         <v>83</v>
       </c>
       <c r="I14" s="50" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="60">
-      <c r="A15" s="104"/>
-      <c r="B15" s="106"/>
+      <c r="A15" s="107"/>
+      <c r="B15" s="105"/>
       <c r="C15" s="49" t="s">
-        <v>154</v>
-      </c>
-      <c r="D15" s="102"/>
-      <c r="E15" s="102"/>
-      <c r="F15" s="102"/>
+        <v>153</v>
+      </c>
+      <c r="D15" s="101"/>
+      <c r="E15" s="101"/>
+      <c r="F15" s="101"/>
       <c r="G15" s="50" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H15" s="58" t="s">
         <v>4</v>
@@ -3586,28 +3600,28 @@
         <v>12</v>
       </c>
       <c r="B16" s="49" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C16" s="49" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D16" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E16" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F16" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G16" s="50" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H16" s="61" t="s">
         <v>87</v>
       </c>
       <c r="I16" s="59" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="45">
@@ -3618,694 +3632,684 @@
         <v>133</v>
       </c>
       <c r="C17" s="49" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D17" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E17" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F17" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G17" s="50" t="s">
-        <v>162</v>
-      </c>
-      <c r="H17" s="63" t="s">
+        <v>161</v>
+      </c>
+      <c r="H17" s="61" t="s">
         <v>17</v>
       </c>
       <c r="I17" s="50" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="60">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="45">
       <c r="A18" s="49">
-        <v>14</v>
-      </c>
-      <c r="B18" s="49" t="s">
-        <v>134</v>
+        <v>15</v>
+      </c>
+      <c r="B18" s="50" t="s">
+        <v>123</v>
       </c>
       <c r="C18" s="49" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D18" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E18" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F18" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G18" s="50" t="s">
-        <v>163</v>
-      </c>
-      <c r="H18" s="61" t="s">
-        <v>18</v>
+        <v>161</v>
+      </c>
+      <c r="H18" s="63" t="s">
+        <v>17</v>
       </c>
       <c r="I18" s="50" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="45">
       <c r="A19" s="49">
-        <v>15</v>
-      </c>
-      <c r="B19" s="50" t="s">
-        <v>123</v>
+        <v>16</v>
+      </c>
+      <c r="B19" s="49" t="s">
+        <v>81</v>
       </c>
       <c r="C19" s="49" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D19" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E19" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F19" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G19" s="50" t="s">
-        <v>162</v>
-      </c>
-      <c r="H19" s="63" t="s">
+        <v>165</v>
+      </c>
+      <c r="H19" s="58" t="s">
+        <v>37</v>
+      </c>
+      <c r="I19" s="59" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="45">
+      <c r="A20" s="106">
         <v>17</v>
       </c>
-      <c r="I19" s="50" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" ht="45">
-      <c r="A20" s="49">
-        <v>16</v>
-      </c>
-      <c r="B20" s="49" t="s">
-        <v>81</v>
+      <c r="B20" s="104" t="s">
+        <v>112</v>
       </c>
       <c r="C20" s="49" t="s">
         <v>154</v>
       </c>
-      <c r="D20" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="E20" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="F20" s="57" t="s">
-        <v>168</v>
+      <c r="D20" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="E20" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="F20" s="100" t="s">
+        <v>167</v>
       </c>
       <c r="G20" s="50" t="s">
-        <v>166</v>
-      </c>
-      <c r="H20" s="58" t="s">
-        <v>37</v>
-      </c>
-      <c r="I20" s="59" t="s">
-        <v>30</v>
+        <v>161</v>
+      </c>
+      <c r="H20" s="63" t="s">
+        <v>17</v>
+      </c>
+      <c r="I20" s="50" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="45">
-      <c r="A21" s="103">
-        <v>17</v>
-      </c>
-      <c r="B21" s="105" t="s">
-        <v>112</v>
-      </c>
+      <c r="A21" s="107"/>
+      <c r="B21" s="105"/>
       <c r="C21" s="49" t="s">
-        <v>155</v>
-      </c>
-      <c r="D21" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="E21" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="F21" s="101" t="s">
-        <v>168</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="D21" s="101"/>
+      <c r="E21" s="101"/>
+      <c r="F21" s="101"/>
       <c r="G21" s="50" t="s">
-        <v>162</v>
-      </c>
-      <c r="H21" s="63" t="s">
-        <v>17</v>
-      </c>
-      <c r="I21" s="50" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="45">
-      <c r="A22" s="104"/>
-      <c r="B22" s="106"/>
+        <v>165</v>
+      </c>
+      <c r="H21" s="58" t="s">
+        <v>36</v>
+      </c>
+      <c r="I21" s="59" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="60">
+      <c r="A22" s="49">
+        <v>18</v>
+      </c>
+      <c r="B22" s="50" t="s">
+        <v>69</v>
+      </c>
       <c r="C22" s="49" t="s">
-        <v>154</v>
-      </c>
-      <c r="D22" s="102"/>
-      <c r="E22" s="102"/>
-      <c r="F22" s="102"/>
+        <v>153</v>
+      </c>
+      <c r="D22" s="57" t="s">
+        <v>167</v>
+      </c>
+      <c r="E22" s="57" t="s">
+        <v>167</v>
+      </c>
+      <c r="F22" s="57" t="s">
+        <v>167</v>
+      </c>
       <c r="G22" s="50" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="H22" s="58" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="I22" s="59" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" ht="60">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="45">
       <c r="A23" s="49">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B23" s="50" t="s">
-        <v>69</v>
+        <v>104</v>
       </c>
       <c r="C23" s="49" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D23" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E23" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F23" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G23" s="50" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="H23" s="58" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="I23" s="59" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" ht="45">
-      <c r="A24" s="49">
-        <v>19</v>
-      </c>
-      <c r="B24" s="50" t="s">
-        <v>104</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="60">
+      <c r="A24" s="106">
+        <v>20</v>
+      </c>
+      <c r="B24" s="102" t="s">
+        <v>121</v>
       </c>
       <c r="C24" s="49" t="s">
         <v>154</v>
       </c>
-      <c r="D24" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="E24" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="F24" s="57" t="s">
-        <v>168</v>
+      <c r="D24" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="E24" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="F24" s="100" t="s">
+        <v>167</v>
       </c>
       <c r="G24" s="50" t="s">
+        <v>157</v>
+      </c>
+      <c r="H24" s="60" t="s">
+        <v>84</v>
+      </c>
+      <c r="I24" s="50" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="60">
+      <c r="A25" s="107"/>
+      <c r="B25" s="103"/>
+      <c r="C25" s="49" t="s">
+        <v>154</v>
+      </c>
+      <c r="D25" s="101"/>
+      <c r="E25" s="101"/>
+      <c r="F25" s="101"/>
+      <c r="G25" s="50" t="s">
         <v>162</v>
       </c>
-      <c r="H24" s="58" t="s">
-        <v>33</v>
-      </c>
-      <c r="I24" s="59" t="s">
+      <c r="H25" s="61" t="s">
+        <v>18</v>
+      </c>
+      <c r="I25" s="50" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="45">
+      <c r="A26" s="106">
         <v>21</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" ht="60">
-      <c r="A25" s="103">
-        <v>20</v>
-      </c>
-      <c r="B25" s="109" t="s">
-        <v>121</v>
-      </c>
-      <c r="C25" s="49" t="s">
-        <v>155</v>
-      </c>
-      <c r="D25" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="E25" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="F25" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="G25" s="50" t="s">
-        <v>158</v>
-      </c>
-      <c r="H25" s="60" t="s">
-        <v>84</v>
-      </c>
-      <c r="I25" s="50" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="60">
-      <c r="A26" s="104"/>
-      <c r="B26" s="110"/>
+      <c r="B26" s="104" t="s">
+        <v>78</v>
+      </c>
       <c r="C26" s="49" t="s">
         <v>155</v>
       </c>
-      <c r="D26" s="102"/>
-      <c r="E26" s="102"/>
-      <c r="F26" s="102"/>
+      <c r="D26" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="E26" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="F26" s="100" t="s">
+        <v>167</v>
+      </c>
       <c r="G26" s="50" t="s">
+        <v>158</v>
+      </c>
+      <c r="H26" s="58" t="s">
+        <v>56</v>
+      </c>
+      <c r="I26" s="50" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="60">
+      <c r="A27" s="107"/>
+      <c r="B27" s="105"/>
+      <c r="C27" s="49" t="s">
+        <v>153</v>
+      </c>
+      <c r="D27" s="101"/>
+      <c r="E27" s="101"/>
+      <c r="F27" s="101"/>
+      <c r="G27" s="50" t="s">
         <v>163</v>
       </c>
-      <c r="H26" s="61" t="s">
-        <v>18</v>
-      </c>
-      <c r="I26" s="50" t="s">
+      <c r="H27" s="58" t="s">
+        <v>58</v>
+      </c>
+      <c r="I27" s="59" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="60">
+      <c r="A28" s="49">
+        <v>22</v>
+      </c>
+      <c r="B28" s="49" t="s">
+        <v>89</v>
+      </c>
+      <c r="C28" s="49" t="s">
+        <v>153</v>
+      </c>
+      <c r="D28" s="57" t="s">
+        <v>167</v>
+      </c>
+      <c r="E28" s="57" t="s">
+        <v>167</v>
+      </c>
+      <c r="F28" s="57" t="s">
+        <v>167</v>
+      </c>
+      <c r="G28" s="50" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" ht="45">
-      <c r="A27" s="103">
-        <v>21</v>
-      </c>
-      <c r="B27" s="105" t="s">
-        <v>78</v>
-      </c>
-      <c r="C27" s="49" t="s">
-        <v>156</v>
-      </c>
-      <c r="D27" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="E27" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="F27" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="G27" s="50" t="s">
-        <v>159</v>
-      </c>
-      <c r="H27" s="58" t="s">
-        <v>56</v>
-      </c>
-      <c r="I27" s="50" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" ht="60">
-      <c r="A28" s="104"/>
-      <c r="B28" s="106"/>
-      <c r="C28" s="49" t="s">
-        <v>154</v>
-      </c>
-      <c r="D28" s="102"/>
-      <c r="E28" s="102"/>
-      <c r="F28" s="102"/>
-      <c r="G28" s="50" t="s">
-        <v>164</v>
-      </c>
       <c r="H28" s="58" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I28" s="59" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="60">
       <c r="A29" s="49">
-        <v>22</v>
-      </c>
-      <c r="B29" s="49" t="s">
-        <v>89</v>
+        <v>23</v>
+      </c>
+      <c r="B29" s="50" t="s">
+        <v>124</v>
       </c>
       <c r="C29" s="49" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D29" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E29" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F29" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G29" s="50" t="s">
-        <v>164</v>
-      </c>
-      <c r="H29" s="58" t="s">
-        <v>60</v>
+        <v>163</v>
+      </c>
+      <c r="H29" s="60" t="s">
+        <v>87</v>
       </c>
       <c r="I29" s="59" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="60">
-      <c r="A30" s="49">
-        <v>23</v>
-      </c>
-      <c r="B30" s="50" t="s">
-        <v>124</v>
-      </c>
-      <c r="C30" s="49" t="s">
-        <v>156</v>
-      </c>
-      <c r="D30" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="E30" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="F30" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="G30" s="50" t="s">
-        <v>164</v>
-      </c>
-      <c r="H30" s="60" t="s">
-        <v>87</v>
-      </c>
-      <c r="I30" s="59" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" s="88" customFormat="1" ht="48" customHeight="1">
-      <c r="A31" s="84">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" s="88" customFormat="1" ht="48" customHeight="1">
+      <c r="A30" s="84">
         <v>24</v>
       </c>
-      <c r="B31" s="84" t="s">
-        <v>178</v>
-      </c>
-      <c r="C31" s="84" t="s">
-        <v>154</v>
-      </c>
-      <c r="D31" s="85" t="s">
-        <v>168</v>
-      </c>
-      <c r="E31" s="86" t="s">
-        <v>168</v>
-      </c>
-      <c r="F31" s="86" t="s">
-        <v>168</v>
-      </c>
-      <c r="G31" s="62" t="s">
-        <v>166</v>
-      </c>
-      <c r="H31" s="87" t="s">
+      <c r="B30" s="84" t="s">
+        <v>177</v>
+      </c>
+      <c r="C30" s="84" t="s">
+        <v>153</v>
+      </c>
+      <c r="D30" s="85" t="s">
+        <v>167</v>
+      </c>
+      <c r="E30" s="86" t="s">
+        <v>167</v>
+      </c>
+      <c r="F30" s="86" t="s">
+        <v>167</v>
+      </c>
+      <c r="G30" s="62" t="s">
+        <v>165</v>
+      </c>
+      <c r="H30" s="87" t="s">
         <v>31</v>
       </c>
-      <c r="I31" s="62" t="s">
+      <c r="I30" s="62" t="s">
         <v>47</v>
       </c>
     </row>
+    <row r="31" spans="1:9" ht="60">
+      <c r="A31" s="106">
+        <v>25</v>
+      </c>
+      <c r="B31" s="104" t="s">
+        <v>79</v>
+      </c>
+      <c r="C31" s="49" t="s">
+        <v>153</v>
+      </c>
+      <c r="D31" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="E31" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="F31" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="G31" s="50" t="s">
+        <v>162</v>
+      </c>
+      <c r="H31" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="I31" s="59" t="s">
+        <v>25</v>
+      </c>
+    </row>
     <row r="32" spans="1:9" ht="60">
-      <c r="A32" s="103">
-        <v>25</v>
-      </c>
-      <c r="B32" s="105" t="s">
-        <v>79</v>
-      </c>
+      <c r="A32" s="107"/>
+      <c r="B32" s="105"/>
       <c r="C32" s="49" t="s">
         <v>154</v>
       </c>
-      <c r="D32" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="E32" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="F32" s="101" t="s">
-        <v>168</v>
-      </c>
+      <c r="D32" s="101"/>
+      <c r="E32" s="101"/>
+      <c r="F32" s="101"/>
       <c r="G32" s="50" t="s">
         <v>163</v>
       </c>
-      <c r="H32" s="58" t="s">
-        <v>3</v>
+      <c r="H32" s="60" t="s">
+        <v>87</v>
       </c>
       <c r="I32" s="59" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" ht="60">
-      <c r="A33" s="104"/>
-      <c r="B33" s="106"/>
+        <v>163</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="45">
+      <c r="A33" s="49">
+        <v>26</v>
+      </c>
+      <c r="B33" s="50" t="s">
+        <v>117</v>
+      </c>
       <c r="C33" s="49" t="s">
         <v>155</v>
       </c>
-      <c r="D33" s="102"/>
-      <c r="E33" s="102"/>
-      <c r="F33" s="102"/>
+      <c r="D33" s="57" t="s">
+        <v>167</v>
+      </c>
+      <c r="E33" s="57" t="s">
+        <v>167</v>
+      </c>
+      <c r="F33" s="57" t="s">
+        <v>167</v>
+      </c>
       <c r="G33" s="50" t="s">
-        <v>164</v>
-      </c>
-      <c r="H33" s="60" t="s">
-        <v>87</v>
-      </c>
-      <c r="I33" s="59" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" ht="45">
+        <v>156</v>
+      </c>
+      <c r="H33" s="64" t="s">
+        <v>8</v>
+      </c>
+      <c r="I33" s="50" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="60">
       <c r="A34" s="49">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B34" s="50" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="C34" s="49" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D34" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E34" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F34" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G34" s="50" t="s">
+        <v>162</v>
+      </c>
+      <c r="H34" s="58" t="s">
+        <v>5</v>
+      </c>
+      <c r="I34" s="59" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="60">
+      <c r="A35" s="106">
+        <v>28</v>
+      </c>
+      <c r="B35" s="102" t="s">
+        <v>88</v>
+      </c>
+      <c r="C35" s="49" t="s">
+        <v>155</v>
+      </c>
+      <c r="D35" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="E35" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="F35" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="G35" s="50" t="s">
         <v>157</v>
       </c>
-      <c r="H34" s="64" t="s">
-        <v>8</v>
-      </c>
-      <c r="I34" s="50" t="s">
+      <c r="H35" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="I35" s="50" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="60">
-      <c r="A35" s="49">
-        <v>27</v>
-      </c>
-      <c r="B35" s="50" t="s">
-        <v>110</v>
-      </c>
-      <c r="C35" s="49" t="s">
-        <v>154</v>
-      </c>
-      <c r="D35" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="E35" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="F35" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="G35" s="50" t="s">
+    <row r="36" spans="1:9" ht="60">
+      <c r="A36" s="107"/>
+      <c r="B36" s="103"/>
+      <c r="C36" s="49" t="s">
+        <v>153</v>
+      </c>
+      <c r="D36" s="101"/>
+      <c r="E36" s="101"/>
+      <c r="F36" s="101"/>
+      <c r="G36" s="50" t="s">
         <v>163</v>
       </c>
-      <c r="H35" s="58" t="s">
-        <v>5</v>
-      </c>
-      <c r="I35" s="59" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="60">
-      <c r="A36" s="103">
-        <v>28</v>
-      </c>
-      <c r="B36" s="109" t="s">
-        <v>88</v>
-      </c>
-      <c r="C36" s="49" t="s">
-        <v>156</v>
-      </c>
-      <c r="D36" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="E36" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="F36" s="101" t="s">
-        <v>168</v>
-      </c>
-      <c r="G36" s="50" t="s">
+      <c r="H36" s="58" t="s">
+        <v>59</v>
+      </c>
+      <c r="I36" s="59" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="45">
+      <c r="A37" s="49">
+        <v>29</v>
+      </c>
+      <c r="B37" s="51" t="s">
+        <v>71</v>
+      </c>
+      <c r="C37" s="49" t="s">
+        <v>153</v>
+      </c>
+      <c r="D37" s="57" t="s">
+        <v>167</v>
+      </c>
+      <c r="E37" s="57" t="s">
+        <v>167</v>
+      </c>
+      <c r="F37" s="57" t="s">
+        <v>167</v>
+      </c>
+      <c r="G37" s="50" t="s">
         <v>158</v>
       </c>
-      <c r="H36" s="61" t="s">
-        <v>84</v>
-      </c>
-      <c r="I36" s="50" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" ht="60">
-      <c r="A37" s="104"/>
-      <c r="B37" s="110"/>
-      <c r="C37" s="49" t="s">
-        <v>154</v>
-      </c>
-      <c r="D37" s="102"/>
-      <c r="E37" s="102"/>
-      <c r="F37" s="102"/>
-      <c r="G37" s="50" t="s">
-        <v>164</v>
-      </c>
       <c r="H37" s="58" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="I37" s="59" t="s">
-        <v>45</v>
+        <v>86</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="45">
       <c r="A38" s="49">
-        <v>29</v>
-      </c>
-      <c r="B38" s="51" t="s">
-        <v>71</v>
+        <v>30</v>
+      </c>
+      <c r="B38" s="49" t="s">
+        <v>132</v>
       </c>
       <c r="C38" s="49" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="D38" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E38" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F38" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G38" s="50" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H38" s="58" t="s">
-        <v>54</v>
-      </c>
-      <c r="I38" s="59" t="s">
-        <v>86</v>
+        <v>56</v>
+      </c>
+      <c r="I38" s="50" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="45">
       <c r="A39" s="49">
-        <v>30</v>
-      </c>
-      <c r="B39" s="49" t="s">
-        <v>132</v>
+        <v>31</v>
+      </c>
+      <c r="B39" s="48" t="s">
+        <v>126</v>
       </c>
       <c r="C39" s="49" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="D39" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E39" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F39" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G39" s="50" t="s">
-        <v>159</v>
-      </c>
-      <c r="H39" s="58" t="s">
-        <v>56</v>
+        <v>165</v>
+      </c>
+      <c r="H39" s="63" t="s">
+        <v>61</v>
       </c>
       <c r="I39" s="50" t="s">
-        <v>43</v>
+        <v>165</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="45">
       <c r="A40" s="49">
-        <v>31</v>
-      </c>
-      <c r="B40" s="48" t="s">
-        <v>126</v>
+        <v>32</v>
+      </c>
+      <c r="B40" s="50" t="s">
+        <v>96</v>
       </c>
       <c r="C40" s="49" t="s">
+        <v>153</v>
+      </c>
+      <c r="D40" s="57" t="s">
+        <v>167</v>
+      </c>
+      <c r="E40" s="57" t="s">
+        <v>167</v>
+      </c>
+      <c r="F40" s="57" t="s">
+        <v>167</v>
+      </c>
+      <c r="G40" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="H40" s="56" t="s">
+        <v>11</v>
+      </c>
+      <c r="I40" s="89" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="60">
+      <c r="A41" s="106">
+        <v>33</v>
+      </c>
+      <c r="B41" s="104" t="s">
+        <v>75</v>
+      </c>
+      <c r="C41" s="49" t="s">
         <v>155</v>
       </c>
-      <c r="D40" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="E40" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="F40" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="G40" s="50" t="s">
-        <v>166</v>
-      </c>
-      <c r="H40" s="63" t="s">
-        <v>61</v>
-      </c>
-      <c r="I40" s="50" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="45">
-      <c r="A41" s="49">
-        <v>32</v>
-      </c>
-      <c r="B41" s="50" t="s">
-        <v>96</v>
-      </c>
-      <c r="C41" s="49" t="s">
-        <v>154</v>
-      </c>
-      <c r="D41" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="E41" s="57" t="s">
-        <v>168</v>
-      </c>
-      <c r="F41" s="57" t="s">
-        <v>168</v>
+      <c r="D41" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="E41" s="100" t="s">
+        <v>167</v>
+      </c>
+      <c r="F41" s="100" t="s">
+        <v>167</v>
       </c>
       <c r="G41" s="50" t="s">
-        <v>157</v>
-      </c>
-      <c r="H41" s="56" t="s">
-        <v>11</v>
-      </c>
-      <c r="I41" s="92" t="s">
-        <v>15</v>
+        <v>162</v>
+      </c>
+      <c r="H41" s="61" t="s">
+        <v>18</v>
+      </c>
+      <c r="I41" s="50" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="42" spans="1:9" ht="60">
-      <c r="A42" s="90">
-        <v>33</v>
-      </c>
-      <c r="B42" s="91" t="s">
-        <v>75</v>
-      </c>
+      <c r="A42" s="107"/>
+      <c r="B42" s="105"/>
       <c r="C42" s="49" t="s">
-        <v>165</v>
-      </c>
-      <c r="D42" s="89" t="s">
-        <v>168</v>
-      </c>
-      <c r="E42" s="89" t="s">
-        <v>168</v>
-      </c>
-      <c r="F42" s="89" t="s">
-        <v>168</v>
-      </c>
+        <v>164</v>
+      </c>
+      <c r="D42" s="101"/>
+      <c r="E42" s="101"/>
+      <c r="F42" s="101"/>
       <c r="G42" s="50" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H42" s="58" t="s">
         <v>29</v>
@@ -4322,19 +4326,19 @@
         <v>102</v>
       </c>
       <c r="C43" s="49" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D43" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E43" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F43" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G43" s="50" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H43" s="58" t="s">
         <v>56</v>
@@ -4351,19 +4355,19 @@
         <v>72</v>
       </c>
       <c r="C44" s="49" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D44" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E44" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F44" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G44" s="50" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H44" s="58" t="s">
         <v>32</v>
@@ -4380,19 +4384,19 @@
         <v>64</v>
       </c>
       <c r="C45" s="49" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D45" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E45" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F45" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G45" s="50" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H45" s="56" t="s">
         <v>9</v>
@@ -4409,19 +4413,19 @@
         <v>67</v>
       </c>
       <c r="C46" s="49" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D46" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E46" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F46" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G46" s="50" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H46" s="58" t="s">
         <v>49</v>
@@ -4437,40 +4441,21 @@
   <sortState ref="B2:I39">
     <sortCondition ref="B1"/>
   </sortState>
-  <mergeCells count="40">
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="F36:F37"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="E32:E33"/>
-    <mergeCell ref="F32:F33"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="E21:E22"/>
+  <mergeCells count="45">
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="D41:D42"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="F41:F42"/>
     <mergeCell ref="F14:F15"/>
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="B4:B5"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="F26:F27"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="A26:A27"/>
     <mergeCell ref="D11:D12"/>
     <mergeCell ref="E11:E12"/>
     <mergeCell ref="F11:F12"/>
@@ -4478,6 +4463,30 @@
     <mergeCell ref="A11:A12"/>
     <mergeCell ref="B14:B15"/>
     <mergeCell ref="A14:A15"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="B31:B32"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>